<commit_message>
More boxplot changes. Nonparametric analysis unfinished
</commit_message>
<xml_diff>
--- a/open_loop_results/open_loop_margins.xlsx
+++ b/open_loop_results/open_loop_margins.xlsx
@@ -895,7 +895,7 @@
         <v>2.121469186808064</v>
       </c>
       <c r="E16" t="n">
-        <v>379.2000990850913</v>
+        <v>19.20009908509132</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
@@ -903,7 +903,7 @@
         <v>2.121469186808064</v>
       </c>
       <c r="I16" t="n">
-        <v>379.2000990850913</v>
+        <v>19.20009908509132</v>
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
@@ -1069,7 +1069,7 @@
         <v>2.215322031492847</v>
       </c>
       <c r="E22" t="n">
-        <v>380.0662043257428</v>
+        <v>20.06620432574283</v>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
@@ -1077,7 +1077,7 @@
         <v>2.215322031492847</v>
       </c>
       <c r="I22" t="n">
-        <v>380.0662043257428</v>
+        <v>20.06620432574283</v>
       </c>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
@@ -1156,7 +1156,7 @@
         <v>2.702353198656887</v>
       </c>
       <c r="E25" t="n">
-        <v>382.9995968134995</v>
+        <v>22.99959681349947</v>
       </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
@@ -1243,7 +1243,7 @@
         <v>2.477582878890399</v>
       </c>
       <c r="E28" t="n">
-        <v>389.0924066176296</v>
+        <v>29.09240661762965</v>
       </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
@@ -1251,7 +1251,7 @@
         <v>2.477582878890399</v>
       </c>
       <c r="I28" t="n">
-        <v>389.0924066176296</v>
+        <v>29.09240661762965</v>
       </c>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr"/>

</xml_diff>